<commit_message>
Bump version to 1.0.2 (add external functions help references)
</commit_message>
<xml_diff>
--- a/inst/extdata/Demografia_Castor_canadensis_results.xlsx
+++ b/inst/extdata/Demografia_Castor_canadensis_results.xlsx
@@ -1,41 +1,85 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dpala\Documents\StablePopulation\inst\extdata\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD85CB0D-D6F1-4B79-86EC-500603AA1DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t>Population Profile</t>
-  </si>
-  <si>
-    <t>alpha</t>
-  </si>
-  <si>
-    <t>beta</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+  <si>
+    <t xml:space="preserve">Population Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alpha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.03111851556499</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.373515897948223</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.248401215459375</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.181642560977468</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.139514126020067</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.110574263418846</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0896139264290044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0738645774713443</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0617031638416951</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0521107440568469</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0444142767434909</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0381513341633812</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0329940199584531</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0287037407608105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0251030882365365</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -71,15 +115,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -361,15 +396,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="25.36328125" customWidth="1"/>
-    <col min="2" max="2" width="18.81640625" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -380,89 +411,117 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1.03111851556499</v>
-      </c>
-      <c r="C2">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>0.37351589794822299</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>0.24840121545937499</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>0.181642560977468</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>0.13951412602006699</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>0.11057426341884601</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>8.9613926429004398E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>7.3864577471344298E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10">
-        <v>6.1703163841695101E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11">
-        <v>5.2110744056846903E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12">
-        <v>4.4414276743490903E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13">
-        <v>3.8151334163381199E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14">
-        <v>3.2994019958453101E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15">
-        <v>2.87037407608105E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16">
-        <v>2.5103088236536501E-2</v>
-      </c>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3"/>
+      <c r="C3"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4"/>
+      <c r="C4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5"/>
+      <c r="C5"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6"/>
+      <c r="C6"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7"/>
+      <c r="C7"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8"/>
+      <c r="C8"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9"/>
+      <c r="C9"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10"/>
+      <c r="C10"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11"/>
+      <c r="C11"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12"/>
+      <c r="C12"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13"/>
+      <c r="C13"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14"/>
+      <c r="C14"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15"/>
+      <c r="C15"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16"/>
+      <c r="C16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>